<commit_message>
feat: auto-reload budget when Excel file is updated
</commit_message>
<xml_diff>
--- a/data/2026 New Monthly Budge.xlsx
+++ b/data/2026 New Monthly Budge.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp-my.sharepoint.com/personal/alan_chiu_hp_com/Documents/Project/AL Budget/預算/Power bi new/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CHIUAL\Documents\budget_app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{7A51C465-FE13-4502-A833-D8A59771F2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF014A2E-898A-4907-AEE1-9CB9B599B971}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F0F391-E610-4E23-B5D2-6C250BB82754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC45FCFC-8C40-4023-96F5-06A5E3DCB0EC}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC45FCFC-8C40-4023-96F5-06A5E3DCB0EC}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 New Monthly budge_Alan" sheetId="2" r:id="rId1"/>
@@ -384,9 +384,6 @@
     <t>主食</t>
   </si>
   <si>
-    <t>房租</t>
-  </si>
-  <si>
     <t>大寶養育基金</t>
   </si>
   <si>
@@ -394,6 +391,9 @@
   </si>
   <si>
     <t>交流通訊</t>
+  </si>
+  <si>
+    <t>房貸支出_伯爵</t>
   </si>
 </sst>
 </file>
@@ -897,15 +897,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88F55F1E-EB8D-4A53-B063-F444AEA412CB}">
   <dimension ref="A1:E77"/>
-  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="9.19921875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="4" customWidth="1"/>
     <col min="2" max="2" width="12.5" style="4" customWidth="1"/>
     <col min="3" max="3" width="18" style="4" customWidth="1"/>
-    <col min="4" max="4" width="17.296875" style="4" customWidth="1"/>
-    <col min="5" max="5" width="11.3984375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="11.4140625" style="4" customWidth="1"/>
     <col min="6" max="6" width="10" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.796875" style="4"/>
+    <col min="7" max="16384" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -980,17 +980,17 @@
       <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>113</v>
+      <c r="B5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>116</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="14">
-        <v>30000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1491,7 +1491,7 @@
         <v>9</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>55</v>
@@ -1508,7 +1508,7 @@
         <v>9</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>56</v>
@@ -1525,7 +1525,7 @@
         <v>9</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>57</v>
@@ -1542,7 +1542,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>58</v>
@@ -1559,7 +1559,7 @@
         <v>9</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>59</v>
@@ -1664,7 +1664,7 @@
         <v>17</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -1885,7 +1885,7 @@
         <v>18</v>
       </c>
       <c r="C58" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1895,19 +1895,19 @@
       </c>
     </row>
     <row r="59" spans="1:5">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C59" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="D59" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E59" s="6">
+      <c r="E59" s="8">
         <v>2000</v>
       </c>
     </row>
@@ -2220,17 +2220,18 @@
   </sheetData>
   <autoFilter ref="A1:E77" xr:uid="{88F55F1E-EB8D-4A53-B063-F444AEA412CB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D26C39-EF28-4B76-89D4-1E3E10533B70}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="12.8984375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="8.796875" style="4"/>
+    <col min="1" max="1" width="12.9140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="23.08203125" style="4" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2331,7 +2332,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>80</v>
@@ -2339,7 +2340,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>81</v>
@@ -2347,7 +2348,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>65</v>
@@ -2355,7 +2356,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>66</v>

</xml_diff>